<commit_message>
fix: restore product SKU on the delivery note export
The old client-side DeliveryNotePDF button showed each line's product
SKU under the description; the first cut of the server template
dropped it. GetDeliveryLineItems now joins products.sku, and the
template's item table gets a dedicated SKU column (blank on a
free-text line or an unset SKU).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RJ1QcRJZ9C1WCAVsFGeRw
</commit_message>
<xml_diff>
--- a/db/templates/delivery_default.xlsx
+++ b/db/templates/delivery_default.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
     <t>{{organization.name}}</t>
   </si>
@@ -65,12 +65,18 @@
     <t>Description</t>
   </si>
   <si>
+    <t>SKU</t>
+  </si>
+  <si>
     <t>Quantity</t>
   </si>
   <si>
     <t>{{lineItems.description}}</t>
   </si>
   <si>
+    <t>{{lineItems.sku}}</t>
+  </si>
+  <si>
     <t>{{lineItems.quantity}} {{lineItems.unit}}</t>
   </si>
   <si>
@@ -228,6 +234,9 @@
   </si>
   <si>
     <t>Line item description</t>
+  </si>
+  <si>
+    <t>Linked product's SKU, blank on a free-text line or an unset SKU</t>
   </si>
   <si>
     <t>{{lineItems.quantity}}</t>
@@ -616,8 +625,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="3" min="1" width="20"/>
-    <col customWidth="true" max="4" min="4" width="16"/>
+    <col customWidth="true" max="1" min="1" width="24"/>
+    <col customWidth="true" max="4" min="2" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,31 +699,36 @@
         <v>15</v>
       </c>
       <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="C13" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="D13" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
   </mergeCells>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -731,20 +745,20 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>15</v>
@@ -752,47 +766,47 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11">
@@ -800,71 +814,71 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20">
@@ -872,113 +886,121 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="C31" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="s">
-        <v>74</v>
+      <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="34">
-      <c r="B34" t="s">
-        <v>75</v>
-      </c>
-      <c r="C34" t="s">
-        <v>76</v>
+      <c r="A34" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -986,7 +1008,7 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A34:C34"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>